<commit_message>
Remove em dashes from generated copy and a few UI strings
Descriptions: sentence-2 template used " — " to join the family
character phrase and the gender/concentration clause; now two plain
sentences instead. Regenerated etl/Perfume_Inventory_100.xlsx and
update_descriptions.sql.

Also cleaned up the handful of em dashes in copy written earlier this
session (cart warning/note, checkout note, order confirmation blurb,
checkout error message, the price/brand-name empty-value fallbacks) --
left the pre-existing site title and code comments alone since neither
is generated customer-facing prose.
</commit_message>
<xml_diff>
--- a/etl/Perfume_Inventory_100.xlsx
+++ b/etl/Perfume_Inventory_100.xlsx
@@ -663,7 +663,7 @@
       </c>
       <c r="O3" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot and pepper, moves through sichuan pepper and lavender, settles into ambroxan and cedar. Sharp and green-tinged, built for movement — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with bergamot and pepper, moves through sichuan pepper and lavender, settles into ambroxan and cedar. Sharp and green-tinged, built for movement. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="O4" s="17" t="inlineStr">
         <is>
-          <t>Opens with grapefruit, lemon and mint, moves through ginger and nutmeg, settles into incense and cedar. Smooth and confident, fills a room quietly — an easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
+          <t>Opens with grapefruit, lemon and mint, moves through ginger and nutmeg, settles into incense and cedar. Smooth and confident, fills a room quietly. An easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="O5" s="17" t="inlineStr">
         <is>
-          <t>Opens with pineapple, bergamot and blackcurrant, moves through birch and patchouli, settles into musk and oakmoss. Structured and sophisticated, rewards a second sniff — a confident one-bottle-does-it-all choice, concentrated enough to carry into the evening.</t>
+          <t>Opens with pineapple, bergamot and blackcurrant, moves through birch and patchouli, settles into musk and oakmoss. Structured and sophisticated, rewards a second sniff. A confident one-bottle-does-it-all choice, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
       </c>
       <c r="O6" s="17" t="inlineStr">
         <is>
-          <t>Opens with grapefruit, mint and blood mandarin, moves through rose and cinnamon, settles into leather and amber. Rich and enveloping, built for cooler nights — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with grapefruit, mint and blood mandarin, moves through rose and cinnamon, settles into leather and amber. Rich and enveloping, built for cooler nights. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="O7" s="17" t="inlineStr">
         <is>
-          <t>Opens with grapefruit and marine notes, moves through bay leaf and jasmine, settles into guaiac wood and oakmoss. Sharp and green-tinged, built for movement — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with grapefruit and marine notes, moves through bay leaf and jasmine, settles into guaiac wood and oakmoss. Sharp and green-tinged, built for movement. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="O8" s="17" t="inlineStr">
         <is>
-          <t>Opens with mint, green apple and lemon, moves through tonka bean and geranium, settles into madagascar vanilla and cedar. Herbal and crisp, with a peppery, energetic edge — a dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with mint, green apple and lemon, moves through tonka bean and geranium, settles into madagascar vanilla and cedar. Herbal and crisp, with a peppery, energetic edge. A dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="O9" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, grapefruit and fig leaf, moves through violet leaf and papyrus, settles into musk and tonka. Brisk and confident, the classic aromatic snap — a confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with bergamot, grapefruit and fig leaf, moves through violet leaf and papyrus, settles into musk and tonka. Brisk and confident, the classic aromatic snap. A confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="O10" s="17" t="inlineStr">
         <is>
-          <t>Opens with lavender, moves through iris and ambrette, settles into vetiver and cedar. Smooth and confident, fills a room quietly — an easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
+          <t>Opens with lavender, moves through iris and ambrette, settles into vetiver and cedar. Smooth and confident, fills a room quietly. An easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="O11" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, neroli and green tangerine, moves through jasmine and sea notes, settles into patchouli and cedar. Clean and breezy, the fragrance equivalent of an open window — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with bergamot, neroli and green tangerine, moves through jasmine and sea notes, settles into patchouli and cedar. Clean and breezy, the fragrance equivalent of an open window. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1293,7 @@
       </c>
       <c r="O12" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot and sea notes, moves through geranium and sage, settles into incense and patchouli. Cool and marine, like sea spray on skin — a dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with bergamot and sea notes, moves through geranium and sage, settles into incense and patchouli. Cool and marine, like sea spray on skin. A dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="O13" s="17" t="inlineStr">
         <is>
-          <t>Opens with cardamom and bergamot, moves through lavender and cedar, settles into vetiver and coumarin. Spiced and sensual, the kind of scent people lean in for — a confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with cardamom and bergamot, moves through lavender and cedar, settles into vetiver and coumarin. Spiced and sensual, the kind of scent people lean in for. A confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="O14" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, ginger and sage, moves through juniper and geranium, settles into amberwood and tonka. Sharp and green-tinged, built for movement — an easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
+          <t>Opens with bergamot, ginger and sage, moves through juniper and geranium, settles into amberwood and tonka. Sharp and green-tinged, built for movement. An easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="O15" s="17" t="inlineStr">
         <is>
-          <t>Opens with mint, lavender and bergamot, moves through cinnamon and cumin, settles into vanilla and tonka. Crisp and herbal with a soapy, clean-shaven finish — a confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with mint, lavender and bergamot, moves through cinnamon and cumin, settles into vanilla and tonka. Crisp and herbal with a soapy, clean-shaven finish. A confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="O16" s="17" t="inlineStr">
         <is>
-          <t>Opens with cardamom and mint, moves through lavender, settles into vanilla and tonka bean. Warm and resinous, glowing rather than shouting — a dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with cardamom and mint, moves through lavender, settles into vanilla and tonka bean. Warm and resinous, glowing rather than shouting. A dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="O17" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot and pepper, moves through lavender and coumarin, settles into ambroxan and patchouli. Sharp and green-tinged, built for movement — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with bergamot and pepper, moves through lavender and coumarin, settles into ambroxan and patchouli. Sharp and green-tinged, built for movement. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="O18" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, pink pepper and clary sage, moves through leather and vetiver, settles into patchouli and ambroxan. Smooth and confident, fills a room quietly — an easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
+          <t>Opens with bergamot, pink pepper and clary sage, moves through leather and vetiver, settles into patchouli and ambroxan. Smooth and confident, fills a room quietly. An easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="O19" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, lavender and pineapple, moves through red apple and rose, settles into tonka and sandalwood. Crisp and herbal with a soapy, clean-shaven finish — a confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with bergamot, lavender and pineapple, moves through red apple and rose, settles into tonka and sandalwood. Crisp and herbal with a soapy, clean-shaven finish. A confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -1853,7 +1853,7 @@
       </c>
       <c r="O20" s="17" t="inlineStr">
         <is>
-          <t>Opens with lemon, bergamot and pineapple, moves through jasmine and cyclamen, settles into musk and oakmoss. Sunlit and clean, never heavy — a confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with lemon, bergamot and pineapple, moves through jasmine and cyclamen, settles into musk and oakmoss. Sunlit and clean, never heavy. A confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1923,7 @@
       </c>
       <c r="O21" s="17" t="inlineStr">
         <is>
-          <t>Opens with lemon, ginger and mint, moves through cardamom and lavender, settles into tonka and amberwood. Rich and enveloping, built for cooler nights — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with lemon, ginger and mint, moves through cardamom and lavender, settles into tonka and amberwood. Rich and enveloping, built for cooler nights. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="O22" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot and white pepper, moves through cedar and sage, settles into tonka and cacao. Spiced and sensual, the kind of scent people lean in for — a confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with bergamot and white pepper, moves through cedar and sage, settles into tonka and cacao. Spiced and sensual, the kind of scent people lean in for. A confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="O23" s="17" t="inlineStr">
         <is>
-          <t>Opens with lime, passion fruit and pepper, moves through vodka and ginger, settles into amber and leather. Rich and enveloping, built for cooler nights — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with lime, passion fruit and pepper, moves through vodka and ginger, settles into amber and leather. Rich and enveloping, built for cooler nights. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="O24" s="17" t="inlineStr">
         <is>
-          <t>Opens with grapefruit, coriander and basil, moves through cardamom and ginger, settles into tobacco and amber. Spiced and sensual, the kind of scent people lean in for — a confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with grapefruit, coriander and basil, moves through cardamom and ginger, settles into tobacco and amber. Spiced and sensual, the kind of scent people lean in for. A confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -2203,7 +2203,7 @@
       </c>
       <c r="O25" s="17" t="inlineStr">
         <is>
-          <t>Opens with grapefruit, bergamot and mandarin, moves through pepper and rosemary, settles into musk and incense. Bright and zesty from the first spray, effervescent rather than sweet — a dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with grapefruit, bergamot and mandarin, moves through pepper and rosemary, settles into musk and incense. Bright and zesty from the first spray, effervescent rather than sweet. A dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="O26" s="17" t="inlineStr">
         <is>
-          <t>Opens with rosewood, cardamom and sichuan pepper, moves through oud and sandalwood, settles into tonka bean and vanilla. Warm and grounded, built around a real wood backbone — built to wear well on anyone, concentrated enough to carry into the evening.</t>
+          <t>Opens with rosewood, cardamom and sichuan pepper, moves through oud and sandalwood, settles into tonka bean and vanilla. Warm and grounded, built around a real wood backbone. Built to wear well on anyone, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="O27" s="17" t="inlineStr">
         <is>
-          <t>Opens with tobacco leaf and spices, moves through vanilla and cacao, settles into dried fruits and woody notes. Warm and resinous, glowing rather than shouting — built to wear well on anyone, concentrated enough to carry into the evening.</t>
+          <t>Opens with tobacco leaf and spices, moves through vanilla and cacao, settles into dried fruits and woody notes. Warm and resinous, glowing rather than shouting. Built to wear well on anyone, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -2413,7 +2413,7 @@
       </c>
       <c r="O28" s="17" t="inlineStr">
         <is>
-          <t>Opens with cardamom, moves through leather and jasmine, settles into amber and moss. Smoky and supple, real leather rather than an idea of it — built to wear well on anyone, concentrated enough to carry into the evening.</t>
+          <t>Opens with cardamom, moves through leather and jasmine, settles into amber and moss. Smoky and supple, real leather rather than an idea of it. Built to wear well on anyone, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="O29" s="17" t="inlineStr">
         <is>
-          <t>Opens with mandarin, cardamom and saffron, moves through orange blossom and kulfi, settles into amber and sandalwood. Spiced and sensual, the kind of scent people lean in for — a confident one-bottle-does-it-all choice, concentrated enough to carry into the evening.</t>
+          <t>Opens with mandarin, cardamom and saffron, moves through orange blossom and kulfi, settles into amber and sandalwood. Spiced and sensual, the kind of scent people lean in for. A confident one-bottle-does-it-all choice, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="O30" s="17" t="inlineStr">
         <is>
-          <t>Opens with spices and rum, moves through tuberose and iris, settles into tonka and benzoin. Warm and resinous, glowing rather than shouting — a dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with spices and rum, moves through tuberose and iris, settles into tonka and benzoin. Warm and resinous, glowing rather than shouting. A dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="O31" s="17" t="inlineStr">
         <is>
-          <t>Opens with orange, bergamot and mandarin, moves through rose and jasmine, settles into patchouli and vetiver. Earthy and refined, with real depth to it — an easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
+          <t>Opens with orange, bergamot and mandarin, moves through rose and jasmine, settles into patchouli and vetiver. Earthy and refined, with real depth to it. An easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="O32" s="17" t="inlineStr">
         <is>
-          <t>Opens with aldehydes, neroli and ylang-ylang, moves through rose and jasmine, settles into sandalwood and vanilla. Delicate but never quiet, a bouquet that lingers — an easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
+          <t>Opens with aldehydes, neroli and ylang-ylang, moves through rose and jasmine, settles into sandalwood and vanilla. Delicate but never quiet, a bouquet that lingers. An easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
       </c>
       <c r="O33" s="17" t="inlineStr">
         <is>
-          <t>Opens with grapefruit and quince, moves through jasmine and hyacinth, settles into amber and white musk. Delicate but never quiet, a bouquet that lingers — an easy, wear-anywhere choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with grapefruit and quince, moves through jasmine and hyacinth, settles into amber and white musk. Delicate but never quiet, a bouquet that lingers. An easy, wear-anywhere choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="O34" s="17" t="inlineStr">
         <is>
-          <t>Opens with pear, melon and magnolia, moves through rose and jasmine, settles into musk and vanilla. Romantic and airy, blooming outward as it wears — a confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
+          <t>Opens with pear, melon and magnolia, moves through rose and jasmine, settles into musk and vanilla. Romantic and airy, blooming outward as it wears. A confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="O35" s="17" t="inlineStr">
         <is>
-          <t>Opens with blood orange and mandarin, moves through grasse rose and peony, settles into rosewood and patchouli. Soft-petaled and radiant, built around a true floral heart — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with blood orange and mandarin, moves through grasse rose and peony, settles into rosewood and patchouli. Soft-petaled and radiant, built around a true floral heart. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="O36" s="17" t="inlineStr">
         <is>
-          <t>Opens with blackcurrant and pear, moves through iris and jasmine, settles into praline and vanilla. Sweet and edible without tipping into dessert — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with blackcurrant and pear, moves through iris and jasmine, settles into praline and vanilla. Sweet and edible without tipping into dessert. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -3043,7 +3043,7 @@
       </c>
       <c r="O37" s="17" t="inlineStr">
         <is>
-          <t>Opens with pink pepper, orange blossom and pear, moves through coffee and jasmine, settles into vanilla and patchouli. Sweet and edible without tipping into dessert — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with pink pepper, orange blossom and pear, moves through coffee and jasmine, settles into vanilla and patchouli. Sweet and edible without tipping into dessert. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="O38" s="17" t="inlineStr">
         <is>
-          <t>Opens with mandarin, lavender and blackcurrant, moves through lavender and orange blossom, settles into vanilla and musk. Soft-petaled and radiant, built around a true floral heart — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with mandarin, lavender and blackcurrant, moves through lavender and orange blossom, settles into vanilla and musk. Soft-petaled and radiant, built around a true floral heart. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="O39" s="17" t="inlineStr">
         <is>
-          <t>Opens with tea, bergamot and osmanthus, moves through jasmine and orchid, settles into patchouli and musk. Soft-petaled and radiant, built around a true floral heart — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with tea, bergamot and osmanthus, moves through jasmine and orchid, settles into patchouli and musk. Soft-petaled and radiant, built around a true floral heart. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -3253,7 +3253,7 @@
       </c>
       <c r="O40" s="17" t="inlineStr">
         <is>
-          <t>Opens with almond, coffee and bergamot, moves through tuberose and jasmine, settles into tonka and cacao. Rich and enveloping, built for cooler nights — an easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
+          <t>Opens with almond, coffee and bergamot, moves through tuberose and jasmine, settles into tonka and cacao. Rich and enveloping, built for cooler nights. An easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="O41" s="17" t="inlineStr">
         <is>
-          <t>Opens with strawberry, violet leaf and grapefruit, moves through jasmine and gardenia, settles into musk and vanilla. Romantic and airy, blooming outward as it wears — a confident one-bottle-does-it-all pick, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with strawberry, violet leaf and grapefruit, moves through jasmine and gardenia, settles into musk and vanilla. Romantic and airy, blooming outward as it wears. A confident one-bottle-does-it-all pick, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -3393,7 +3393,7 @@
       </c>
       <c r="O42" s="17" t="inlineStr">
         <is>
-          <t>Opens with bitter orange, raspberry and neroli, moves through orange blossom and jasmine, settles into honey and patchouli. Romantic and airy, blooming outward as it wears — a confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
+          <t>Opens with bitter orange, raspberry and neroli, moves through orange blossom and jasmine, settles into honey and patchouli. Romantic and airy, blooming outward as it wears. A confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="O43" s="17" t="inlineStr">
         <is>
-          <t>Opens with blackcurrant and mandarin, moves through rose and freesia, settles into patchouli and vanilla. Earthy and refined, with real depth to it — an easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
+          <t>Opens with blackcurrant and mandarin, moves through rose and freesia, settles into patchouli and vanilla. Earthy and refined, with real depth to it. An easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="O44" s="17" t="inlineStr">
         <is>
-          <t>Opens with pomegranate, yuzu and ice, moves through peony and magnolia, settles into musk and amber. Romantic and airy, blooming outward as it wears — a confident one-bottle-does-it-all pick, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with pomegranate, yuzu and ice, moves through peony and magnolia, settles into musk and amber. Romantic and airy, blooming outward as it wears. A confident one-bottle-does-it-all pick, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -3603,7 +3603,7 @@
       </c>
       <c r="O45" s="17" t="inlineStr">
         <is>
-          <t>Opens with sicilian lemon, apple and bellflower, moves through bamboo and jasmine, settles into cedar and amber. Sunlit and clean, never heavy — a confident one-bottle-does-it-all pick, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with sicilian lemon, apple and bellflower, moves through bamboo and jasmine, settles into cedar and amber. Sunlit and clean, never heavy. A confident one-bottle-does-it-all pick, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -3673,7 +3673,7 @@
       </c>
       <c r="O46" s="17" t="inlineStr">
         <is>
-          <t>Opens with jasmine, moves through cashmeran and amber, settles into white amber and woody notes. Spiced and sensual, the kind of scent people lean in for — a confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
+          <t>Opens with jasmine, moves through cashmeran and amber, settles into white amber and woody notes. Spiced and sensual, the kind of scent people lean in for. A confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="O47" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, melon and coconut, moves through honey and red berries, settles into vanilla and patchouli. Indulgent and cozy, built around real sweetness — a confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
+          <t>Opens with bergamot, melon and coconut, moves through honey and red berries, settles into vanilla and patchouli. Indulgent and cozy, built around real sweetness. A confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -3813,7 +3813,7 @@
       </c>
       <c r="O48" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, pear and pink pepper, moves through rose and jasmine, settles into white musk and vanilla. Romantic and airy, blooming outward as it wears — a confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
+          <t>Opens with bergamot, pear and pink pepper, moves through rose and jasmine, settles into white musk and vanilla. Romantic and airy, blooming outward as it wears. A confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -3883,7 +3883,7 @@
       </c>
       <c r="O49" s="17" t="inlineStr">
         <is>
-          <t>Opens with neroli and bergamot, moves through jasmine and amber, settles into musk and vanilla. Soft-petaled and radiant, built around a true floral heart — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with neroli and bergamot, moves through jasmine and amber, settles into musk and vanilla. Soft-petaled and radiant, built around a true floral heart. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="O50" s="17" t="inlineStr">
         <is>
-          <t>Opens with blackcurrant, raspberry and blackberry, moves through jasmine and violet, settles into musk and amber. Indulgent and cozy, built around real sweetness — a confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
+          <t>Opens with blackcurrant, raspberry and blackberry, moves through jasmine and violet, settles into musk and amber. Indulgent and cozy, built around real sweetness. A confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="O51" s="17" t="inlineStr">
         <is>
-          <t>Opens with jasmine and tuberose, moves through rangoon creeper and orange blossom, settles into sandalwood and musk. Soft-petaled and radiant, built around a true floral heart — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with jasmine and tuberose, moves through rangoon creeper and orange blossom, settles into sandalwood and musk. Soft-petaled and radiant, built around a true floral heart. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -4093,7 +4093,7 @@
       </c>
       <c r="O52" s="17" t="inlineStr">
         <is>
-          <t>Opens with pear and red berries, moves through gardenia and frangipani, settles into brown sugar and patchouli. Soft-petaled and radiant, built around a true floral heart — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with pear and red berries, moves through gardenia and frangipani, settles into brown sugar and patchouli. Soft-petaled and radiant, built around a true floral heart. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="O53" s="17" t="inlineStr">
         <is>
-          <t>Opens with blood orange and mandarin, moves through honey and gardenia, settles into patchouli and beeswax. Warm and comforting, like something baked — an easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
+          <t>Opens with blood orange and mandarin, moves through honey and gardenia, settles into patchouli and beeswax. Warm and comforting, like something baked. An easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="O54" s="17" t="inlineStr">
         <is>
-          <t>Opens with osmanthus and african orange flower, moves through musk and amber, settles into vanilla and patchouli. Structured and sophisticated, rewards a second sniff — a confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
+          <t>Opens with osmanthus and african orange flower, moves through musk and amber, settles into vanilla and patchouli. Structured and sophisticated, rewards a second sniff. A confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -4303,7 +4303,7 @@
       </c>
       <c r="O55" s="17" t="inlineStr">
         <is>
-          <t>Opens with peony, freesia and litchi, moves through rose and magnolia, settles into cedar and amber. Delicate but never quiet, a bouquet that lingers — an easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
+          <t>Opens with peony, freesia and litchi, moves through rose and magnolia, settles into cedar and amber. Delicate but never quiet, a bouquet that lingers. An easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -4373,7 +4373,7 @@
       </c>
       <c r="O56" s="17" t="inlineStr">
         <is>
-          <t>Opens with lavender, pear and bergamot, moves through whipped cream and praline, settles into musk and woods. Indulgent and cozy, built around real sweetness — a confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
+          <t>Opens with lavender, pear and bergamot, moves through whipped cream and praline, settles into musk and woods. Indulgent and cozy, built around real sweetness. A confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -4443,7 +4443,7 @@
       </c>
       <c r="O57" s="17" t="inlineStr">
         <is>
-          <t>Opens with brown sugar, moves through vanilla and jasmine, settles into musk and tonka. Indulgent and cozy, built around real sweetness — a confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
+          <t>Opens with brown sugar, moves through vanilla and jasmine, settles into musk and tonka. Indulgent and cozy, built around real sweetness. A confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="O58" s="17" t="inlineStr">
         <is>
-          <t>Opens with saffron and jasmine, moves through amberwood and ambergris, settles into fir resin and cedar. Rich and enveloping, built for cooler nights — genuinely unisex, no gendered marketing required, concentrated enough to carry into the evening.</t>
+          <t>Opens with saffron and jasmine, moves through amberwood and ambergris, settles into fir resin and cedar. Rich and enveloping, built for cooler nights. Genuinely unisex, no gendered marketing required, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="O59" s="17" t="inlineStr">
         <is>
-          <t>Opens with cardamom, iris and violet, moves through ambrox and sandalwood, settles into leather and cedar. Dry and textured, more sweater than cologne — flexible enough for any wardrobe, concentrated enough to carry into the evening.</t>
+          <t>Opens with cardamom, iris and violet, moves through ambrox and sandalwood, settles into leather and cedar. Dry and textured, more sweater than cologne. Flexible enough for any wardrobe, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -4653,7 +4653,7 @@
       </c>
       <c r="O60" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, lemon and pepper, moves through incense and pine needles, settles into amber and vanilla. Dry and textured, more sweater than cologne — flexible enough for any wardrobe, concentrated enough to carry into the evening.</t>
+          <t>Opens with bergamot, lemon and pepper, moves through incense and pine needles, settles into amber and vanilla. Dry and textured, more sweater than cologne. Flexible enough for any wardrobe, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -4723,7 +4723,7 @@
       </c>
       <c r="O61" s="17" t="inlineStr">
         <is>
-          <t>Opens with ambrette seeds, moves through sea salt, settles into sage and driftwood. Airy and transparent, built to feel weightless — flexible enough for any wardrobe, a lighter, splashier cut, best refreshed through the day.</t>
+          <t>Opens with ambrette seeds, moves through sea salt, settles into sage and driftwood. Airy and transparent, built to feel weightless. Flexible enough for any wardrobe, a lighter, splashier cut, best refreshed through the day.</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="O62" s="17" t="inlineStr">
         <is>
-          <t>Opens with pear and melon, moves through freesia and rose, settles into patchouli and musk. Soft-petaled and radiant, built around a true floral heart — built to wear well on anyone, a lighter, splashier cut, best refreshed through the day.</t>
+          <t>Opens with pear and melon, moves through freesia and rose, settles into patchouli and musk. Soft-petaled and radiant, built around a true floral heart. Built to wear well on anyone, a lighter, splashier cut, best refreshed through the day.</t>
         </is>
       </c>
     </row>
@@ -4863,7 +4863,7 @@
       </c>
       <c r="O63" s="17" t="inlineStr">
         <is>
-          <t>Opens with pink pepper, neroli and lemon, moves through rum and clary sage, settles into tobacco and vanilla. Warm and resinous, glowing rather than shouting — built to wear well on anyone, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with pink pepper, neroli and lemon, moves through rum and clary sage, settles into tobacco and vanilla. Warm and resinous, glowing rather than shouting. Built to wear well on anyone, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -4933,7 +4933,7 @@
       </c>
       <c r="O64" s="17" t="inlineStr">
         <is>
-          <t>Opens with clove, pink pepper and orange, moves through chestnut and guaiac wood, settles into vanilla and cashmeran. Indulgent and cozy, built around real sweetness — flexible enough for any wardrobe, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with clove, pink pepper and orange, moves through chestnut and guaiac wood, settles into vanilla and cashmeran. Indulgent and cozy, built around real sweetness. Flexible enough for any wardrobe, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="O65" s="17" t="inlineStr">
         <is>
-          <t>Opens with lemon and verbena, moves through violet leaf and iris, settles into sandalwood and ambergris. Crisp and herbal with a soapy, clean-shaven finish — a confident one-bottle-does-it-all choice, concentrated enough to carry into the evening.</t>
+          <t>Opens with lemon and verbena, moves through violet leaf and iris, settles into sandalwood and ambergris. Crisp and herbal with a soapy, clean-shaven finish. A confident one-bottle-does-it-all choice, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="O66" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot and mandarin, moves through green tea and blackcurrant, settles into musk and sandalwood. Clean and breezy, the fragrance equivalent of an open window — genuinely unisex, no gendered marketing required, concentrated enough to carry into the evening.</t>
+          <t>Opens with bergamot and mandarin, moves through green tea and blackcurrant, settles into musk and sandalwood. Clean and breezy, the fragrance equivalent of an open window. Genuinely unisex, no gendered marketing required, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5143,7 @@
       </c>
       <c r="O67" s="17" t="inlineStr">
         <is>
-          <t>Opens with apple, bergamot and lavender, moves through geranium and violet, settles into vanilla and sandalwood. Rich and enveloping, built for cooler nights — an easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
+          <t>Opens with apple, bergamot and lavender, moves through geranium and violet, settles into vanilla and sandalwood. Rich and enveloping, built for cooler nights. An easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="O68" s="17" t="inlineStr">
         <is>
-          <t>Opens with litchi, rhubarb and bergamot, moves through turkish rose and peony, settles into vanilla and musk. Romantic and airy, blooming outward as it wears — a confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
+          <t>Opens with litchi, rhubarb and bergamot, moves through turkish rose and peony, settles into vanilla and musk. Romantic and airy, blooming outward as it wears. A confident one-bottle-does-it-all pick, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -5283,7 +5283,7 @@
       </c>
       <c r="O69" s="17" t="inlineStr">
         <is>
-          <t>Opens with saffron and nutmeg, moves through oud and patchouli, settles into musk and sandalwood. Smooth and confident, fills a room quietly — genuinely unisex, no gendered marketing required, concentrated enough to carry into the evening.</t>
+          <t>Opens with saffron and nutmeg, moves through oud and patchouli, settles into musk and sandalwood. Smooth and confident, fills a room quietly. Genuinely unisex, no gendered marketing required, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -5353,7 +5353,7 @@
       </c>
       <c r="O70" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, lavender and lemon, moves through honey and cinnamon, settles into tonka and vanilla. Warm and resinous, glowing rather than shouting — a dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with bergamot, lavender and lemon, moves through honey and cinnamon, settles into tonka and vanilla. Warm and resinous, glowing rather than shouting. A dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="O71" s="17" t="inlineStr">
         <is>
-          <t>Opens with black pepper, lemon and mandarin, moves through rose and geranium, settles into tonka and vanilla. Spiced and sensual, the kind of scent people lean in for — a confident one-bottle-does-it-all choice, concentrated enough to carry into the evening.</t>
+          <t>Opens with black pepper, lemon and mandarin, moves through rose and geranium, settles into tonka and vanilla. Spiced and sensual, the kind of scent people lean in for. A confident one-bottle-does-it-all choice, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -5493,7 +5493,7 @@
       </c>
       <c r="O72" s="17" t="inlineStr">
         <is>
-          <t>Opens with ginger and bergamot, moves through sage and violet leaf, settles into vetiver and woods. Herbal and crisp, with a peppery, energetic edge — a dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with ginger and bergamot, moves through sage and violet leaf, settles into vetiver and woods. Herbal and crisp, with a peppery, energetic edge. A dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="O73" s="17" t="inlineStr">
         <is>
-          <t>Opens with blackcurrant and jasmine, moves through jasmine and bourbon vanilla, settles into woods and musk. Soft-petaled and radiant, built around a true floral heart — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with blackcurrant and jasmine, moves through jasmine and bourbon vanilla, settles into woods and musk. Soft-petaled and radiant, built around a true floral heart. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="O74" s="17" t="inlineStr">
         <is>
-          <t>Opens with pear, cardamom and iris, moves through iris and lavender, settles into patchouli and leather. Rich and enveloping, built for cooler nights — an easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
+          <t>Opens with pear, cardamom and iris, moves through iris and lavender, settles into patchouli and leather. Rich and enveloping, built for cooler nights. An easy, no-fuss pick for daily wear, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -5703,7 +5703,7 @@
       </c>
       <c r="O75" s="17" t="inlineStr">
         <is>
-          <t>Opens with apple, bergamot and lemon, moves through cinnamon and clove, settles into sandalwood and vetiver. Warm and grounded, built around a real wood backbone — a dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with apple, bergamot and lemon, moves through cinnamon and clove, settles into sandalwood and vetiver. Warm and grounded, built around a real wood backbone. A dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -5773,7 +5773,7 @@
       </c>
       <c r="O76" s="17" t="inlineStr">
         <is>
-          <t>Opens with fresh notes, moves through elemi and ginger, settles into cedar and vanilla. Smooth and confident, fills a room quietly — an easy, no-fuss pick for daily wear, the most concentrated cut here, built to last all day.</t>
+          <t>Opens with fresh notes, moves through elemi and ginger, settles into cedar and vanilla. Smooth and confident, fills a room quietly. An easy, no-fuss pick for daily wear, the most concentrated cut here, built to last all day.</t>
         </is>
       </c>
     </row>
@@ -5843,7 +5843,7 @@
       </c>
       <c r="O77" s="17" t="inlineStr">
         <is>
-          <t>Opens with lemon, bergamot and pineapple, moves through nutmeg and violet, settles into musk and amber. Sunlit and clean, never heavy — flexible enough for any wardrobe, a lighter, splashier cut, best refreshed through the day.</t>
+          <t>Opens with lemon, bergamot and pineapple, moves through nutmeg and violet, settles into musk and amber. Sunlit and clean, never heavy. Flexible enough for any wardrobe, a lighter, splashier cut, best refreshed through the day.</t>
         </is>
       </c>
     </row>
@@ -5913,7 +5913,7 @@
       </c>
       <c r="O78" s="17" t="inlineStr">
         <is>
-          <t>Opens with lavender, mandarin and bergamot, moves through sage and coriander, settles into sandalwood and musk. Structured and cool, a modern take on an old formula — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with lavender, mandarin and bergamot, moves through sage and coriander, settles into sandalwood and musk. Structured and cool, a modern take on an old formula. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="O79" s="17" t="inlineStr">
         <is>
-          <t>Opens with melon, cucumber and mandarin, moves through sage and geranium, settles into musk and suede. Airy and transparent, built to feel weightless — a confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with melon, cucumber and mandarin, moves through sage and geranium, settles into musk and suede. Airy and transparent, built to feel weightless. A confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -6053,7 +6053,7 @@
       </c>
       <c r="O80" s="17" t="inlineStr">
         <is>
-          <t>Opens with cranberry, italian lemon and grapefruit, moves through saffron and sage, settles into amber and cedar. Dry and textured, more sweater than cologne — a confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with cranberry, italian lemon and grapefruit, moves through saffron and sage, settles into amber and cedar. Dry and textured, more sweater than cologne. A confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -6123,7 +6123,7 @@
       </c>
       <c r="O81" s="17" t="inlineStr">
         <is>
-          <t>Opens with neroli, black pepper and cardamom, moves through iris and geranium, settles into amber and patchouli. Delicate but never quiet, a bouquet that lingers — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with neroli, black pepper and cardamom, moves through iris and geranium, settles into amber and patchouli. Delicate but never quiet, a bouquet that lingers. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -6193,7 +6193,7 @@
       </c>
       <c r="O82" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot and ambrette, moves through sage and agarwood, settles into musk and ambroxan. Cool and marine, like sea spray on skin — a dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with bergamot and ambrette, moves through sage and agarwood, settles into musk and ambroxan. Cool and marine, like sea spray on skin. A dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -6263,7 +6263,7 @@
       </c>
       <c r="O83" s="17" t="inlineStr">
         <is>
-          <t>Opens with grapefruit, cardamom and tarragon, moves through birch leaf and nutmeg, settles into vetiver and guaiac wood. Brisk and confident, the classic aromatic snap — a confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with grapefruit, cardamom and tarragon, moves through birch leaf and nutmeg, settles into vetiver and guaiac wood. Brisk and confident, the classic aromatic snap. A confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="O84" s="17" t="inlineStr">
         <is>
-          <t>Opens with yuzu, bergamot and cypress, moves through nutmeg and lily, settles into amber and tobacco. Clean and breezy, the fragrance equivalent of an open window — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with yuzu, bergamot and cypress, moves through nutmeg and lily, settles into amber and tobacco. Clean and breezy, the fragrance equivalent of an open window. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="O85" s="17" t="inlineStr">
         <is>
-          <t>Opens with blackcurrant and mandarin, moves through rose and violet, settles into vanilla and white musk. Delicate but never quiet, a bouquet that lingers — an easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
+          <t>Opens with blackcurrant and mandarin, moves through rose and violet, settles into vanilla and white musk. Delicate but never quiet, a bouquet that lingers. An easy, wear-anywhere choice, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="O86" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, grapefruit and pink pepper, moves through cinnamon and saffron, settles into tobacco and leather. Rich and enveloping, built for cooler nights — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with bergamot, grapefruit and pink pepper, moves through cinnamon and saffron, settles into tobacco and leather. Rich and enveloping, built for cooler nights. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -6543,7 +6543,7 @@
       </c>
       <c r="O87" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot and lemon, moves through olive blossom and star anise, settles into tonka bean and leather. Rich and enveloping, built for cooler nights — an easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with bergamot and lemon, moves through olive blossom and star anise, settles into tonka bean and leather. Rich and enveloping, built for cooler nights. An easy, no-fuss pick for daily wear, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -6613,7 +6613,7 @@
       </c>
       <c r="O88" s="17" t="inlineStr">
         <is>
-          <t>Opens with orange blossom and bergamot, moves through tuberose and indian jasmine, settles into cedar and vanilla. Soft-petaled and radiant, built around a true floral heart — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with orange blossom and bergamot, moves through tuberose and indian jasmine, settles into cedar and vanilla. Soft-petaled and radiant, built around a true floral heart. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -6683,7 +6683,7 @@
       </c>
       <c r="O89" s="17" t="inlineStr">
         <is>
-          <t>Opens with black truffle, ylang-ylang and bergamot, moves through orchid and spices, settles into patchouli and vanilla. Spiced and sensual, the kind of scent people lean in for — flexible enough for any wardrobe, concentrated enough to carry into the evening.</t>
+          <t>Opens with black truffle, ylang-ylang and bergamot, moves through orchid and spices, settles into patchouli and vanilla. Spiced and sensual, the kind of scent people lean in for. Flexible enough for any wardrobe, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -6753,7 +6753,7 @@
       </c>
       <c r="O90" s="17" t="inlineStr">
         <is>
-          <t>Opens with black cherry, cherry liqueur and bitter almond, moves through turkish rose and jasmine, settles into tonka and vanilla. Warm and comforting, like something baked — genuinely unisex, no gendered marketing required, concentrated enough to carry into the evening.</t>
+          <t>Opens with black cherry, cherry liqueur and bitter almond, moves through turkish rose and jasmine, settles into tonka and vanilla. Warm and comforting, like something baked. Genuinely unisex, no gendered marketing required, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -6823,7 +6823,7 @@
       </c>
       <c r="O91" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, neroli and citron, moves through hyacinth and clary sage, settles into musk and cedar. Cool and marine, like sea spray on skin — a dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with bergamot, neroli and citron, moves through hyacinth and clary sage, settles into musk and cedar. Cool and marine, like sea spray on skin. A dependable, everyday men's signature, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -6893,7 +6893,7 @@
       </c>
       <c r="O92" s="17" t="inlineStr">
         <is>
-          <t>Opens with pineapple, bergamot and grapefruit, moves through patchouli and cedar, settles into oakmoss and musk. Structured and sophisticated, rewards a second sniff — flexible enough for any wardrobe, concentrated enough to carry into the evening.</t>
+          <t>Opens with pineapple, bergamot and grapefruit, moves through patchouli and cedar, settles into oakmoss and musk. Structured and sophisticated, rewards a second sniff. Flexible enough for any wardrobe, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -6963,7 +6963,7 @@
       </c>
       <c r="O93" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot, oregano and pepper, moves through amber and cistus, settles into leather and sandalwood. Warm and resinous, glowing rather than shouting — a dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with bergamot, oregano and pepper, moves through amber and cistus, settles into leather and sandalwood. Warm and resinous, glowing rather than shouting. A dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -7033,7 +7033,7 @@
       </c>
       <c r="O94" s="17" t="inlineStr">
         <is>
-          <t>Opens with red apple, moves through peony and jasmine, settles into suede. Delicate but never quiet, a bouquet that lingers — an easy, wear-anywhere choice, a lighter, splashier cut, best refreshed through the day.</t>
+          <t>Opens with red apple, moves through peony and jasmine, settles into suede. Delicate but never quiet, a bouquet that lingers. An easy, wear-anywhere choice, a lighter, splashier cut, best refreshed through the day.</t>
         </is>
       </c>
     </row>
@@ -7103,7 +7103,7 @@
       </c>
       <c r="O95" s="17" t="inlineStr">
         <is>
-          <t>Opens with fig leaf, moves through fig and coconut, settles into fig tree wood and cedar. Grassy and sharp, unmistakably outdoors — flexible enough for any wardrobe, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with fig leaf, moves through fig and coconut, settles into fig tree wood and cedar. Grassy and sharp, unmistakably outdoors. Flexible enough for any wardrobe, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -7173,7 +7173,7 @@
       </c>
       <c r="O96" s="17" t="inlineStr">
         <is>
-          <t>Opens with amber, moves through benzoin and labdanum, settles into vanilla and tonka. Spiced and sensual, the kind of scent people lean in for — flexible enough for any wardrobe, concentrated enough to carry into the evening.</t>
+          <t>Opens with amber, moves through benzoin and labdanum, settles into vanilla and tonka. Spiced and sensual, the kind of scent people lean in for. Flexible enough for any wardrobe, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -7243,7 +7243,7 @@
       </c>
       <c r="O97" s="17" t="inlineStr">
         <is>
-          <t>Opens with peach and champagne rosé, moves through rose, settles into musk. Soft-petaled and radiant, built around a true floral heart — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with peach and champagne rosé, moves through rose, settles into musk. Soft-petaled and radiant, built around a true floral heart. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -7313,7 +7313,7 @@
       </c>
       <c r="O98" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot and pink pepper, moves through iris and cashmere wood, settles into vetiver and haitian vetiver. Dry and textured, more sweater than cologne — a confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
+          <t>Opens with bergamot and pink pepper, moves through iris and cashmere wood, settles into vetiver and haitian vetiver. Dry and textured, more sweater than cologne. A confident one-bottle-does-it-all choice, light enough for daytime, with a few hours of wear.</t>
         </is>
       </c>
     </row>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="O99" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot and lavender, moves through jasmine and iris, settles into vanilla and tonka. Warm and resinous, glowing rather than shouting — a versatile, everyday signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with bergamot and lavender, moves through jasmine and iris, settles into vanilla and tonka. Warm and resinous, glowing rather than shouting. A versatile, everyday signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -7453,7 +7453,7 @@
       </c>
       <c r="O100" s="17" t="inlineStr">
         <is>
-          <t>Opens with cognac, moves through cinnamon and tonka, settles into vanilla and praline. Sweet and edible without tipping into dessert — built to wear well on anyone, concentrated enough to carry into the evening.</t>
+          <t>Opens with cognac, moves through cinnamon and tonka, settles into vanilla and praline. Sweet and edible without tipping into dessert. Built to wear well on anyone, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="O101" s="17" t="inlineStr">
         <is>
-          <t>Opens with cinnamon, nutmeg and cardamom, moves through lavender and licorice, settles into amber and sandalwood. Warm and resinous, glowing rather than shouting — a dependable, everyday men's signature, the most concentrated cut here, built to last all day.</t>
+          <t>Opens with cinnamon, nutmeg and cardamom, moves through lavender and licorice, settles into amber and sandalwood. Warm and resinous, glowing rather than shouting. A dependable, everyday men's signature, the most concentrated cut here, built to last all day.</t>
         </is>
       </c>
     </row>
@@ -7593,7 +7593,7 @@
       </c>
       <c r="O102" s="17" t="inlineStr">
         <is>
-          <t>Opens with bergamot and orange blossom, moves through orange blossom, settles into patchouli and ambrette. Soft-petaled and radiant, built around a true floral heart — a dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
+          <t>Opens with bergamot and orange blossom, moves through orange blossom, settles into patchouli and ambrette. Soft-petaled and radiant, built around a true floral heart. A dependable, everyday men's signature, concentrated enough to carry into the evening.</t>
         </is>
       </c>
     </row>

</xml_diff>